<commit_message>
Improve normalizer, JV engine, models & GUI
Refactor normalizer, engine and model workflow, add inspection/test utilities and GUI file actions. billing_sheet.BillingSheet now validates file existence and uses BillingNormalizer to produce and load the "Normalized" sheet. JVGenerator uses JVEngine to run processing (writes temp normalized file, captures engine rows, builds fallback DataFrame, and delegates final write to the engine). JVEngine posting-key logic/comment corrected and credit posting key sign fixed. Normalizer auto-selects billing sheets, supports non-interactive runs, marks critical/missing/calculated columns, and only computes GL recharge columns when source data is absent. Added CLI/inspection scripts (check_pkey_logic.py, inspect_pkeys.py), a feb comparison test (test_feb_comparison.py), and multiple normalized/output XLSX fixtures. UI (main_gui) gains Open/Locate buttons and handlers to access generated JV files.
</commit_message>
<xml_diff>
--- a/scripts/test_manual_input.xlsx
+++ b/scripts/test_manual_input.xlsx
@@ -1,34 +1,97 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+  <si>
+    <t>Workday ID</t>
+  </si>
+  <si>
+    <t>Classification</t>
+  </si>
+  <si>
+    <t>Billed/ Unbilled</t>
+  </si>
+  <si>
+    <t>Invoice No.</t>
+  </si>
+  <si>
+    <t>EmpNo</t>
+  </si>
+  <si>
+    <t>Capability Center</t>
+  </si>
+  <si>
+    <t>Recharge - Payroll</t>
+  </si>
+  <si>
+    <t>Recharge - Manager</t>
+  </si>
+  <si>
+    <t>Recharge - Leadership</t>
+  </si>
+  <si>
+    <t>Recharge - Desk Cost</t>
+  </si>
+  <si>
+    <t>Recharge - Retirals</t>
+  </si>
+  <si>
+    <t>Mark up</t>
+  </si>
+  <si>
+    <t>W1</t>
+  </si>
+  <si>
+    <t>W2</t>
+  </si>
+  <si>
+    <t>Billable</t>
+  </si>
+  <si>
+    <t>Billed</t>
+  </si>
+  <si>
+    <t>INV1</t>
+  </si>
+  <si>
+    <t>E1</t>
+  </si>
+  <si>
+    <t>E2</t>
+  </si>
+  <si>
+    <t>CC1</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +110,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,177 +404,125 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Workday ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Classification</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Billed/ Unbilled</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Invoice No.</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>EmpNo</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Capability Center</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Recharge - Payroll</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Recharge - Manager</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Recharge - Leadership</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Recharge - Desk Cost</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Recharge - Retirals</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Mark up</t>
-        </is>
+    <row r="1" spans="1:12">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>W1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Billable</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Billed</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>INV1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>CC1</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2">
         <v>100</v>
       </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
         <v>10</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>W2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Billable</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Billed</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>INV1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>E2</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CC1</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3">
         <v>200</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3">
         <v>50</v>
       </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
         <v>20</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>